<commit_message>
Added come Unit test for TorpedoStore class.
</commit_message>
<xml_diff>
--- a/test-data/TestScema.xlsx
+++ b/test-data/TestScema.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Bence\Desktop\SzoftverTechnologiák\se-lab4\test-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B70C4752-5B9C-4812-BF0A-4CC110CCF9B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4128B801-83E6-49B8-A3DF-43FAFD17B818}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{D1D97A60-C7A2-42F2-9DF9-FBD004590D14}"/>
   </bookViews>
@@ -887,6 +887,8 @@
     <col min="7" max="7" width="41.140625" customWidth="1"/>
     <col min="8" max="8" width="35.140625" customWidth="1"/>
     <col min="9" max="9" width="35.85546875" customWidth="1"/>
+    <col min="10" max="10" width="31.85546875" customWidth="1"/>
+    <col min="11" max="11" width="29" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="88.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">

</xml_diff>